<commit_message>
docs(v1.3): integrate governance expansion
- add six new controls and their implementation playbooks
- patch existing controls and refresh documentation, guidance files, and generated assets
- update AI instruction files and validate the release bundle

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/downloads/compliance-officer-checklist.xlsx
+++ b/docs/downloads/compliance-officer-checklist.xlsx
@@ -546,7 +546,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: Compliance Officer  |  FSI Agent Governance Framework v1.2.41 — February 2026</t>
+          <t>Role: Compliance Officer  |  FSI Agent Governance Framework v1.3.0 — March 2026</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>FSI Agent Governance Framework v1.2.41 — February 2026</t>
+          <t>FSI Agent Governance Framework v1.3.0 — March 2026</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CCompliance Officer Checklist</oddHeader>
-    <oddFooter>&amp;CFSI Agent Governance Framework v1.2.41 — February 2026</oddFooter>
+    <oddFooter>&amp;CFSI Agent Governance Framework v1.3.0 — March 2026</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
fix(downloads): bump Excel checklist headers v1.3.0 -> v1.4.0
Drift sweep DIM G finding. All 6 role-based Excel checklists in docs/downloads/ had stale 'FSI Agent Governance Framework v1.3.0 - March 2026' header text (16 cells across 6 files). AMWINS will download these; bumped to v1.4.0 / April 2026 to match site.

Files: compliance-officer, entra-administrator, governance-maturity-dashboard, power-platform-administrator, purview-administrator, sharepoint-administrator.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/downloads/compliance-officer-checklist.xlsx
+++ b/docs/downloads/compliance-officer-checklist.xlsx
@@ -546,7 +546,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: Compliance Officer  |  FSI Agent Governance Framework v1.3.0 — March 2026</t>
+          <t>Role: Compliance Officer  |  FSI Agent Governance Framework v1.4.0 — April 2026</t>
         </is>
       </c>
     </row>
@@ -806,10 +806,11 @@
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="11" t="n"/>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>FSI Agent Governance Framework v1.3.0 — March 2026</t>
+          <t>FSI Agent Governance Framework v1.4.0 — April 2026</t>
         </is>
       </c>
     </row>

</xml_diff>